<commit_message>
demo: use dataset aggregates and EDR area
</commit_message>
<xml_diff>
--- a/data/social-protection/social-protection.xlsx
+++ b/data/social-protection/social-protection.xlsx
@@ -10,6 +10,7 @@
     <sheet name="Households" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Persons" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Enrollments" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="DistrictGeometries" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2040,4 +2041,90 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>district</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>geometry</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>north</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>{"type":"Polygon","coordinates":[[[0,1],[1,1],[1,2],[0,2],[0,1]]]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>south</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>{"type":"Polygon","coordinates":[[[0,-1],[1,-1],[1,0],[0,0],[0,-1]]]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>central</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>{"type":"Polygon","coordinates":[[[0,0],[1,0],[1,1],[0,1],[0,0]]]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>east</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>{"type":"Polygon","coordinates":[[[1,0],[2,0],[2,1],[1,1],[1,0]]]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>west</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>{"type":"Polygon","coordinates":[[[-1,0],[0,0],[0,1],[-1,1],[-1,0]]]}</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Align registry lab demo identifiers
</commit_message>
<xml_diff>
--- a/data/social-protection/social-protection.xlsx
+++ b/data/social-protection/social-protection.xlsx
@@ -489,10 +489,10 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H2" t="n">
         <v>0</v>
@@ -523,10 +523,10 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H3" t="n">
         <v>0</v>
@@ -591,10 +591,10 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G5" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H5" t="n">
         <v>0</v>
@@ -625,13 +625,13 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G6" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="H6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -651,21 +651,21 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>72</v>
+        <v>38</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>not_eligible</t>
+          <t>priority</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -676,27 +676,27 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>NID-2002</t>
+          <t>NID-1008</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>south</t>
+          <t>west</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>priority</t>
+          <t>standard</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="G8" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="H8" t="n">
         <v>0</v>
@@ -710,12 +710,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>NID-2008</t>
+          <t>NID-1010</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>west</t>
+          <t>central</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -727,10 +727,10 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="G9" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="H9" t="n">
         <v>0</v>
@@ -747,7 +747,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G28"/>
+  <dimension ref="A1:G32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -809,7 +809,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="F2" t="b">
         <v>1</v>
@@ -823,7 +823,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>PER-2001</t>
+          <t>PER-1007</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -833,16 +833,16 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>NID-2001</t>
+          <t>NID-1007</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>caregiver</t>
+          <t>grandparent</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>31</v>
+        <v>68</v>
       </c>
       <c r="F3" t="b">
         <v>1</v>
@@ -856,7 +856,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>PER-3001</t>
+          <t>PER-2001</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -866,16 +866,16 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>NID-3001</t>
+          <t>NID-2001</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>sibling</t>
+          <t>caregiver</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>10</v>
+        <v>42</v>
       </c>
       <c r="F4" t="b">
         <v>1</v>
@@ -889,7 +889,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>PER-3002</t>
+          <t>PER-3001</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -899,7 +899,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>NID-3002</t>
+          <t>NID-3001</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -908,54 +908,54 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F5" t="b">
         <v>1</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>hearing</t>
+          <t>none</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>PER-1002</t>
+          <t>PER-3002</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>HH-200</t>
+          <t>HH-100</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>NID-1002</t>
+          <t>NID-3002</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>child</t>
+          <t>sibling</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="F6" t="b">
         <v>1</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>hearing</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>PER-2002</t>
+          <t>PER-1002</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -965,16 +965,16 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>NID-2002</t>
+          <t>NID-1002</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>caregiver</t>
+          <t>child</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>35</v>
+        <v>8</v>
       </c>
       <c r="F7" t="b">
         <v>1</v>
@@ -988,7 +988,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>PER-3003</t>
+          <t>PER-2002</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -998,56 +998,56 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>NID-3003</t>
+          <t>NID-2002</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>grandparent</t>
+          <t>caregiver</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>68</v>
+        <v>38</v>
       </c>
       <c r="F8" t="b">
         <v>1</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>physical</t>
+          <t>none</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>PER-1003</t>
+          <t>PER-3003</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>HH-300</t>
+          <t>HH-200</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>NID-1003</t>
+          <t>NID-3003</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>adult</t>
+          <t>caregiver</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>69</v>
+        <v>35</v>
       </c>
       <c r="F9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>physical</t>
+          <t>none</t>
         </is>
       </c>
     </row>
@@ -1059,7 +1059,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>HH-300</t>
+          <t>HH-200</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1069,11 +1069,11 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>spouse</t>
+          <t>sibling</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>66</v>
+        <v>12</v>
       </c>
       <c r="F10" t="b">
         <v>1</v>
@@ -1087,59 +1087,59 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>PER-1004</t>
+          <t>PER-1003</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>HH-400</t>
+          <t>HH-300</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>NID-1004</t>
+          <t>NID-1003</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>child</t>
+          <t>adult</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>5</v>
+        <v>69</v>
       </c>
       <c r="F11" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>physical</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>PER-2004</t>
+          <t>PER-3005</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>HH-400</t>
+          <t>HH-300</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>NID-2004</t>
+          <t>NID-3005</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>caregiver</t>
+          <t>spouse</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>38</v>
+        <v>66</v>
       </c>
       <c r="F12" t="b">
         <v>1</v>
@@ -1153,7 +1153,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>PER-3005</t>
+          <t>PER-1004</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1163,7 +1163,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>NID-3005</t>
+          <t>NID-1004</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1172,7 +1172,7 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="F13" t="b">
         <v>1</v>
@@ -1186,7 +1186,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>PER-3006</t>
+          <t>PER-2004</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1196,30 +1196,30 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>NID-3006</t>
+          <t>NID-2004</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>child</t>
+          <t>caregiver</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>12</v>
+        <v>38</v>
       </c>
       <c r="F14" t="b">
         <v>1</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>visual</t>
+          <t>none</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>PER-3007</t>
+          <t>PER-3006</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1229,16 +1229,16 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>NID-3007</t>
+          <t>NID-3006</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>grandparent</t>
+          <t>sibling</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>71</v>
+        <v>15</v>
       </c>
       <c r="F15" t="b">
         <v>1</v>
@@ -1252,26 +1252,26 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>PER-1005</t>
+          <t>PER-3007</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>HH-500</t>
+          <t>HH-400</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>NID-1005</t>
+          <t>NID-3007</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>child</t>
+          <t>sibling</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="F16" t="b">
         <v>1</v>
@@ -1285,7 +1285,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>PER-2005</t>
+          <t>PER-1005</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1295,16 +1295,16 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>NID-2005</t>
+          <t>NID-1005</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>caregiver</t>
+          <t>child</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>41</v>
+        <v>13</v>
       </c>
       <c r="F17" t="b">
         <v>1</v>
@@ -1318,7 +1318,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>PER-3008</t>
+          <t>PER-2005</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1328,30 +1328,30 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>NID-3008</t>
+          <t>NID-2005</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>adult</t>
+          <t>caregiver</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>74</v>
+        <v>48</v>
       </c>
       <c r="F18" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>physical</t>
+          <t>none</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>PER-3009</t>
+          <t>PER-3008</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1361,16 +1361,16 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>NID-3009</t>
+          <t>NID-3008</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>sibling</t>
+          <t>caregiver</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>15</v>
+        <v>44</v>
       </c>
       <c r="F19" t="b">
         <v>1</v>
@@ -1384,26 +1384,26 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>PER-1006</t>
+          <t>PER-3009</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>HH-600</t>
+          <t>HH-500</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>NID-1006</t>
+          <t>NID-3009</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>child</t>
+          <t>sibling</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="F20" t="b">
         <v>1</v>
@@ -1417,29 +1417,29 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>PER-2006</t>
+          <t>PER-3010</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>HH-600</t>
+          <t>HH-500</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>NID-2006</t>
+          <t>NID-3010</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>caregiver</t>
+          <t>sibling</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>43</v>
+        <v>16</v>
       </c>
       <c r="F21" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
@@ -1450,26 +1450,26 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>PER-2010</t>
+          <t>PER-3011</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>HH-700</t>
+          <t>HH-500</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>NID-2010</t>
+          <t>NID-3011</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>caregiver</t>
+          <t>sibling</t>
         </is>
       </c>
       <c r="E22" t="n">
-        <v>33</v>
+        <v>9</v>
       </c>
       <c r="F22" t="b">
         <v>1</v>
@@ -1483,17 +1483,17 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>PER-2011</t>
+          <t>PER-1006</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>HH-700</t>
+          <t>HH-600</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>NID-2011</t>
+          <t>NID-1006</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1502,40 +1502,40 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="F23" t="b">
         <v>1</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>physical</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>PER-2012</t>
+          <t>PER-2006</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>HH-700</t>
+          <t>HH-600</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>NID-2012</t>
+          <t>NID-2006</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>child</t>
+          <t>caregiver</t>
         </is>
       </c>
       <c r="E24" t="n">
-        <v>4</v>
+        <v>48</v>
       </c>
       <c r="F24" t="b">
         <v>1</v>
@@ -1549,40 +1549,40 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>PER-2013</t>
+          <t>PER-3012</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>HH-700</t>
+          <t>HH-600</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>NID-2013</t>
+          <t>NID-3012</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>child</t>
+          <t>caregiver</t>
         </is>
       </c>
       <c r="E25" t="n">
-        <v>6</v>
+        <v>45</v>
       </c>
       <c r="F25" t="b">
         <v>1</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>cognitive</t>
+          <t>none</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>PER-2014</t>
+          <t>PER-1008</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1592,16 +1592,16 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>NID-2014</t>
+          <t>NID-1008</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>child</t>
+          <t>single_adult</t>
         </is>
       </c>
       <c r="E26" t="n">
-        <v>9</v>
+        <v>72</v>
       </c>
       <c r="F26" t="b">
         <v>1</v>
@@ -1615,26 +1615,26 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>PER-2015</t>
+          <t>PER-1010</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>HH-700</t>
+          <t>HH-800</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>NID-2015</t>
+          <t>NID-1010</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>adult</t>
+          <t>caregiver</t>
         </is>
       </c>
       <c r="E27" t="n">
-        <v>29</v>
+        <v>55</v>
       </c>
       <c r="F27" t="b">
         <v>1</v>
@@ -1648,7 +1648,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>PER-2008</t>
+          <t>PER-1009</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1658,21 +1658,153 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>NID-2008</t>
+          <t>NID-1009</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>single_adult</t>
+          <t>adult</t>
         </is>
       </c>
       <c r="E28" t="n">
-        <v>41</v>
+        <v>28</v>
       </c>
       <c r="F28" t="b">
         <v>1</v>
       </c>
       <c r="G28" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>PER-3013</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>HH-800</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>NID-3013</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>household_member</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>50</v>
+      </c>
+      <c r="F29" t="b">
+        <v>1</v>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>PER-3014</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>HH-800</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>NID-3014</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>household_member</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>45</v>
+      </c>
+      <c r="F30" t="b">
+        <v>1</v>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>PER-3015</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>HH-800</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>NID-3015</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>child</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>14</v>
+      </c>
+      <c r="F31" t="b">
+        <v>1</v>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>PER-3016</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>HH-800</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>NID-3016</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>child</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>10</v>
+      </c>
+      <c r="F32" t="b">
+        <v>1</v>
+      </c>
+      <c r="G32" t="inlineStr">
         <is>
           <t>none</t>
         </is>
@@ -1689,7 +1821,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1947,16 +2079,16 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>CHILD_SUPPORT</t>
+          <t>DISABILITY_SUPPORT</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>suspended</t>
+          <t>active</t>
         </is>
       </c>
       <c r="G7" t="n">
-        <v>0</v>
+        <v>175</v>
       </c>
       <c r="H7" s="1" t="n">
         <v>45646</v>
@@ -1970,31 +2102,31 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>HH-700</t>
+          <t>HH-100</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>PER-2011</t>
+          <t>PER-1007</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>NID-2011</t>
+          <t>NID-1007</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>CHILD_SUPPORT</t>
+          <t>ELDERLY_PENSION</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>inactive</t>
         </is>
       </c>
       <c r="G8" t="n">
-        <v>140</v>
+        <v>0</v>
       </c>
       <c r="H8" s="1" t="n">
         <v>45901</v>
@@ -2008,34 +2140,110 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>HH-800</t>
+          <t>HH-700</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>PER-2008</t>
+          <t>PER-1008</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>NID-2008</t>
+          <t>NID-1008</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>HEALTH_LINKED_SUPPORT</t>
+          <t>ELDERLY_PENSION</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>inactive</t>
+          <t>active</t>
         </is>
       </c>
       <c r="G9" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="H9" s="1" t="n">
         <v>45751</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>ENR-900</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>HH-800</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>PER-1009</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>NID-1009</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>COMMUNITY_REGISTRY</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" s="1" t="n">
+        <v>45778</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>ENR-1000</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>HH-800</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>PER-1010</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>NID-1010</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>COMMUNITY_REGISTRY</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="G11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" s="1" t="n">
+        <v>45778</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refresh social protection attestation demo
</commit_message>
<xml_diff>
--- a/data/social-protection/social-protection.xlsx
+++ b/data/social-protection/social-protection.xlsx
@@ -10,7 +10,15 @@
     <sheet name="Households" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Persons" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Enrollments" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="DistrictGeometries" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="GroupMemberships" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="SocioEconomicProfiles" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="ScoringEvents" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Programs" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Entitlements" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="PaymentEvents" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="FunctioningProfiles" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="DisabilityDeterminations" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="DistrictGeometries" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -741,6 +749,397 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>profile_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>person_id</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>national_id</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>instrument_code</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>administration_date</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>respondent_relationship</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>domain_severities</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>disability_identifier_met</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>domains_triggering_identifier</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>source_version</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>FUNC-1006</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>PER-1006</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>NID-1006</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>WG-SS-2025</t>
+        </is>
+      </c>
+      <c r="E2" s="1" t="n">
+        <v>45996</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>caregiver</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>mobility=severe;self_care=moderate</t>
+        </is>
+      </c>
+      <c r="H2" t="b">
+        <v>1</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>mobility;self_care</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>2025.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>FUNC-1003</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>PER-1003</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>NID-1003</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>WG-SS-2025</t>
+        </is>
+      </c>
+      <c r="E3" s="1" t="n">
+        <v>45809</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>self</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>mobility=severe</t>
+        </is>
+      </c>
+      <c r="H3" t="b">
+        <v>1</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>mobility</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>2025.2</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>determination_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>person_id</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>national_id</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>authority</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>determination_status</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>support_category</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>valid_from</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>valid_until</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>review_due</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>DIS-1006</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>PER-1006</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>NID-1006</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Disability Assessment Authority</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>top_up</t>
+        </is>
+      </c>
+      <c r="G2" s="1" t="n">
+        <v>46011</v>
+      </c>
+      <c r="H2" s="1" t="n">
+        <v>46376</v>
+      </c>
+      <c r="I2" s="1" t="n">
+        <v>46315</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>DIS-1003</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>PER-1003</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>NID-1003</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Disability Assessment Authority</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>closed_deceased</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="G3" s="1" t="n">
+        <v>45809</v>
+      </c>
+      <c r="H3" s="1" t="n">
+        <v>45963</v>
+      </c>
+      <c r="I3" s="1" t="n">
+        <v>45963</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>district</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>geometry</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>north</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>{"type":"Polygon","coordinates":[[[0,1],[1,1],[1,2],[0,2],[0,1]]]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>south</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>{"type":"Polygon","coordinates":[[[0,-1],[1,-1],[1,0],[0,0],[0,-1]]]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>central</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>{"type":"Polygon","coordinates":[[[0,0],[1,0],[1,1],[0,1],[0,0]]]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>east</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>{"type":"Polygon","coordinates":[[[1,0],[2,0],[2,1],[1,1],[1,0]]]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>west</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>{"type":"Polygon","coordinates":[[[-1,0],[0,0],[0,1],[-1,1],[-1,0]]]}</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -2257,79 +2656,2490 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:G32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>district</t>
+          <t>membership_id</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>geometry</t>
+          <t>household_id</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>person_id</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>relationship_type</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>start_date</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>end_date</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>membership_status</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>north</t>
+          <t>GM-1001</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>{"type":"Polygon","coordinates":[[[0,1],[1,1],[1,2],[0,2],[0,1]]]}</t>
+          <t>HH-100</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>PER-1001</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>child</t>
+        </is>
+      </c>
+      <c r="E2" s="1" t="n">
+        <v>45658</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>active</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>south</t>
+          <t>GM-1007</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>{"type":"Polygon","coordinates":[[[0,-1],[1,-1],[1,0],[0,0],[0,-1]]]}</t>
+          <t>HH-100</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>PER-1007</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>grandparent</t>
+        </is>
+      </c>
+      <c r="E3" s="1" t="n">
+        <v>45658</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>active</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>central</t>
+          <t>GM-2001</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>{"type":"Polygon","coordinates":[[[0,0],[1,0],[1,1],[0,1],[0,0]]]}</t>
+          <t>HH-100</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>PER-2001</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>caregiver</t>
+        </is>
+      </c>
+      <c r="E4" s="1" t="n">
+        <v>45658</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>active</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>east</t>
+          <t>GM-3001</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>{"type":"Polygon","coordinates":[[[1,0],[2,0],[2,1],[1,1],[1,0]]]}</t>
+          <t>HH-100</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>PER-3001</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>sibling</t>
+        </is>
+      </c>
+      <c r="E5" s="1" t="n">
+        <v>45658</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>active</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>west</t>
+          <t>GM-3002</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>{"type":"Polygon","coordinates":[[[-1,0],[0,0],[0,1],[-1,1],[-1,0]]]}</t>
-        </is>
+          <t>HH-100</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>PER-3002</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>sibling</t>
+        </is>
+      </c>
+      <c r="E6" s="1" t="n">
+        <v>45658</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>GM-1002</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>HH-200</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>PER-1002</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>child</t>
+        </is>
+      </c>
+      <c r="E7" s="1" t="n">
+        <v>45658</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>GM-2002</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>HH-200</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>PER-2002</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>caregiver</t>
+        </is>
+      </c>
+      <c r="E8" s="1" t="n">
+        <v>45658</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>GM-3003</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>HH-200</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>PER-3003</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>caregiver</t>
+        </is>
+      </c>
+      <c r="E9" s="1" t="n">
+        <v>45658</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>GM-3004</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>HH-200</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>PER-3004</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>sibling</t>
+        </is>
+      </c>
+      <c r="E10" s="1" t="n">
+        <v>45658</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>GM-1003</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>HH-300</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>PER-1003</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>adult</t>
+        </is>
+      </c>
+      <c r="E11" s="1" t="n">
+        <v>45658</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>ended_deceased</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>GM-3005</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>HH-300</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>PER-3005</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>spouse</t>
+        </is>
+      </c>
+      <c r="E12" s="1" t="n">
+        <v>45658</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>GM-1004</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>HH-400</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>PER-1004</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>child</t>
+        </is>
+      </c>
+      <c r="E13" s="1" t="n">
+        <v>45658</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>GM-2004</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>HH-400</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>PER-2004</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>caregiver</t>
+        </is>
+      </c>
+      <c r="E14" s="1" t="n">
+        <v>45658</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>GM-3006</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>HH-400</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>PER-3006</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>sibling</t>
+        </is>
+      </c>
+      <c r="E15" s="1" t="n">
+        <v>45658</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>GM-3007</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>HH-400</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>PER-3007</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>sibling</t>
+        </is>
+      </c>
+      <c r="E16" s="1" t="n">
+        <v>45658</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>GM-1005</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>HH-500</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>PER-1005</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>child</t>
+        </is>
+      </c>
+      <c r="E17" s="1" t="n">
+        <v>45658</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>GM-2005</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>HH-500</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>PER-2005</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>caregiver</t>
+        </is>
+      </c>
+      <c r="E18" s="1" t="n">
+        <v>45658</v>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>GM-3008</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>HH-500</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>PER-3008</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>caregiver</t>
+        </is>
+      </c>
+      <c r="E19" s="1" t="n">
+        <v>45658</v>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>GM-3009</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>HH-500</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>PER-3009</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>sibling</t>
+        </is>
+      </c>
+      <c r="E20" s="1" t="n">
+        <v>45658</v>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>GM-3010</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>HH-500</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>PER-3010</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>sibling</t>
+        </is>
+      </c>
+      <c r="E21" s="1" t="n">
+        <v>45658</v>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>GM-3011</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>HH-500</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>PER-3011</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>sibling</t>
+        </is>
+      </c>
+      <c r="E22" s="1" t="n">
+        <v>45658</v>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>GM-1006</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>HH-600</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>PER-1006</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>child</t>
+        </is>
+      </c>
+      <c r="E23" s="1" t="n">
+        <v>45658</v>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>GM-2006</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>HH-600</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>PER-2006</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>caregiver</t>
+        </is>
+      </c>
+      <c r="E24" s="1" t="n">
+        <v>45658</v>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>GM-3012</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>HH-600</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>PER-3012</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>caregiver</t>
+        </is>
+      </c>
+      <c r="E25" s="1" t="n">
+        <v>45658</v>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>GM-1008</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>HH-700</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>PER-1008</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>single_adult</t>
+        </is>
+      </c>
+      <c r="E26" s="1" t="n">
+        <v>45658</v>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>GM-1010</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>HH-800</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>PER-1010</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>caregiver</t>
+        </is>
+      </c>
+      <c r="E27" s="1" t="n">
+        <v>45658</v>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>GM-1009</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>HH-800</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>PER-1009</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>adult</t>
+        </is>
+      </c>
+      <c r="E28" s="1" t="n">
+        <v>45658</v>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>GM-3013</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>HH-800</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>PER-3013</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>household_member</t>
+        </is>
+      </c>
+      <c r="E29" s="1" t="n">
+        <v>45658</v>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>GM-3014</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>HH-800</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>PER-3014</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>household_member</t>
+        </is>
+      </c>
+      <c r="E30" s="1" t="n">
+        <v>45658</v>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>GM-3015</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>HH-800</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>PER-3015</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>child</t>
+        </is>
+      </c>
+      <c r="E31" s="1" t="n">
+        <v>45658</v>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>GM-3016</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>HH-800</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>PER-3016</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>child</t>
+        </is>
+      </c>
+      <c r="E32" s="1" t="n">
+        <v>45658</v>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>profile_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>household_id</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>observation_date</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>instrument</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>collected_by</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>source_version</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>profile_status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>SEP-100</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>HH-100</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="n">
+        <v>45992</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>PMT-CHILD-2025</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>municipal_social_worker</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>2025.4</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>SEP-200</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>HH-200</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="n">
+        <v>45976</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>PMT-CHILD-2025</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>municipal_social_worker</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>2025.4</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>SEP-300</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>HH-300</t>
+        </is>
+      </c>
+      <c r="C4" s="1" t="n">
+        <v>45931</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>PMT-ADULT-2025</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>central_review_team</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>2025.3</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>SEP-400</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>HH-400</t>
+        </is>
+      </c>
+      <c r="C5" s="1" t="n">
+        <v>46001</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>PMT-CHILD-2025</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>municipal_social_worker</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>2025.4</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>SEP-500</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>HH-500</t>
+        </is>
+      </c>
+      <c r="C6" s="1" t="n">
+        <v>45301</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>PMT-CHILD-2024</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>municipal_social_worker</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>2024.1</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>stale</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>SEP-600</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>HH-600</t>
+        </is>
+      </c>
+      <c r="C7" s="1" t="n">
+        <v>45996</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>PMT-DISABILITY-2025</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>assessment_registry</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>2025.4</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>SEP-700</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>HH-700</t>
+        </is>
+      </c>
+      <c r="C8" s="1" t="n">
+        <v>45717</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>PMT-ELDERLY-2025</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>municipal_social_worker</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>2025.2</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>SEP-800</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>HH-800</t>
+        </is>
+      </c>
+      <c r="C9" s="1" t="n">
+        <v>45839</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>PMT-COMMUNITY-2025</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>central_review_team</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>2025.2</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>scoring_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>profile_id</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>scoring_rule</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>scoring_version</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>score_band</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>valid_from</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>valid_until</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>scoring_status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>SCOR-100</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>SEP-100</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>child-benefit-priority</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2025.4</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>priority</t>
+        </is>
+      </c>
+      <c r="F2" s="1" t="n">
+        <v>45992</v>
+      </c>
+      <c r="G2" s="1" t="n">
+        <v>46357</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>SCOR-200</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>SEP-200</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>child-benefit-standard</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>2025.4</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+      <c r="F3" s="1" t="n">
+        <v>45976</v>
+      </c>
+      <c r="G3" s="1" t="n">
+        <v>46341</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>SCOR-300</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>SEP-300</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>death-review</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>2025.3</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>not_eligible</t>
+        </is>
+      </c>
+      <c r="F4" s="1" t="n">
+        <v>45931</v>
+      </c>
+      <c r="G4" s="1" t="n">
+        <v>46296</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>SCOR-400</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>SEP-400</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>child-benefit-priority</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>2025.4</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>priority</t>
+        </is>
+      </c>
+      <c r="F5" s="1" t="n">
+        <v>46001</v>
+      </c>
+      <c r="G5" s="1" t="n">
+        <v>46366</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>SCOR-500</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>SEP-500</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>child-benefit-standard</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>2024.1</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+      <c r="F6" s="1" t="n">
+        <v>45301</v>
+      </c>
+      <c r="G6" s="1" t="n">
+        <v>45667</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>stale</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>SCOR-600</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>SEP-600</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>disability-top-up</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>2025.4</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>priority</t>
+        </is>
+      </c>
+      <c r="F7" s="1" t="n">
+        <v>45996</v>
+      </c>
+      <c r="G7" s="1" t="n">
+        <v>46361</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>SCOR-700</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>SEP-700</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>elderly-pension</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>2025.2</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>standard</t>
+        </is>
+      </c>
+      <c r="F8" s="1" t="n">
+        <v>45717</v>
+      </c>
+      <c r="G8" s="1" t="n">
+        <v>46022</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>expired</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>SCOR-800</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>SEP-800</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>community-review</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>2025.2</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>not_eligible</t>
+        </is>
+      </c>
+      <c r="F9" s="1" t="n">
+        <v>45839</v>
+      </c>
+      <c r="G9" s="1" t="n">
+        <v>46204</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>policy_denied</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>program_code</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>display_name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>authority</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>benefit_type</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>CHILD_SUPPORT</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Child Support Grant</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Social Protection Authority</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>cash_transfer</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>HEALTH_LINKED_SUPPORT</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Health-Linked Support</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Social Protection Authority</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>conditional_cash_transfer</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>DISABILITY_SUPPORT</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Disability Support Top-Up</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Disability Assessment Authority</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>cash_top_up</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>ELDERLY_PENSION</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Elderly Pension</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Social Protection Authority</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>pension</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>COMMUNITY_REGISTRY</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Community Registry</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Social Registry Authority</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>registry_only</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>entitlement_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>enrollment_id</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>benefit_modality</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>amount</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>amount_band</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>currency</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>coverage_start</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>coverage_end</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>entitlement_status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>ENT-100</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>ENR-100</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>cash</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>85.5</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>standard_child</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G2" s="1" t="n">
+        <v>46023</v>
+      </c>
+      <c r="H2" s="1" t="n">
+        <v>46387</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>ENT-200</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>ENR-200</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>cash</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G3" s="1" t="n">
+        <v>45352</v>
+      </c>
+      <c r="H3" s="1" t="n">
+        <v>45657</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>inactive</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>ENT-300</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>ENR-300</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>cash</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>review</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G4" s="1" t="n">
+        <v>45809</v>
+      </c>
+      <c r="H4" s="1" t="n">
+        <v>46173</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>review_required</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>ENT-400</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ENR-400</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>cash</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>110</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>priority_child</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G5" s="1" t="n">
+        <v>46023</v>
+      </c>
+      <c r="H5" s="1" t="n">
+        <v>46387</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>ENT-500</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ENR-500</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>cash</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>60</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>standard_child</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G6" s="1" t="n">
+        <v>45658</v>
+      </c>
+      <c r="H6" s="1" t="n">
+        <v>46022</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>stale_source</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>ENT-600</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ENR-600</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>cash</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>175</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>disability_top_up</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G7" s="1" t="n">
+        <v>46023</v>
+      </c>
+      <c r="H7" s="1" t="n">
+        <v>46387</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>ENT-700</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>ENR-700</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>cash</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>elderly_pension</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G8" s="1" t="n">
+        <v>45901</v>
+      </c>
+      <c r="H8" s="1" t="n">
+        <v>46022</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>expired</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>ENT-800</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>ENR-800</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>cash</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>100</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>elderly_pension</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G9" s="1" t="n">
+        <v>46023</v>
+      </c>
+      <c r="H9" s="1" t="n">
+        <v>46387</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>ENT-900</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>ENR-900</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G10" s="1" t="n">
+        <v>45778</v>
+      </c>
+      <c r="H10" s="1" t="n">
+        <v>46143</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>policy_denied</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>payment_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>entitlement_id</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>cycle</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>delivery_channel</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>payment_date</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>reconciled</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>PAY-100-JAN</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>ENT-100</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>paid</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>mobile_money</t>
+        </is>
+      </c>
+      <c r="F2" s="1" t="n">
+        <v>46037</v>
+      </c>
+      <c r="G2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>PAY-400-JAN</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>ENT-400</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>paid</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>bank_transfer</t>
+        </is>
+      </c>
+      <c r="F3" s="1" t="n">
+        <v>46037</v>
+      </c>
+      <c r="G3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>PAY-500-DEC</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>ENT-500</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>held_stale_profile</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>mobile_money</t>
+        </is>
+      </c>
+      <c r="F4" s="1" t="n">
+        <v>46006</v>
+      </c>
+      <c r="G4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>PAY-600-JAN</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ENT-600</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>paid</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>cash_agent</t>
+        </is>
+      </c>
+      <c r="F5" s="1" t="n">
+        <v>46038</v>
+      </c>
+      <c r="G5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>PAY-700-JAN</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ENT-700</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>not_paid_expired</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>cash_agent</t>
+        </is>
+      </c>
+      <c r="F6" s="1" t="n">
+        <v>46038</v>
+      </c>
+      <c r="G6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>PAY-900-JAN</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ENT-900</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>not_paid_policy_denied</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="F7" s="1" t="n">
+        <v>46038</v>
+      </c>
+      <c r="G7" t="b">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Prove evidence gateway release flow
</commit_message>
<xml_diff>
--- a/data/social-protection/social-protection.xlsx
+++ b/data/social-protection/social-protection.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -741,6 +741,40 @@
         <v>6</v>
       </c>
       <c r="H9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>HH-900</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>NID-1011</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>south</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>28</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>priority</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>3</v>
+      </c>
+      <c r="G10" t="n">
+        <v>3</v>
+      </c>
+      <c r="H10" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1146,7 +1180,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G32"/>
+  <dimension ref="A1:G33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2204,6 +2238,39 @@
         <v>1</v>
       </c>
       <c r="G32" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>PER-1011</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>HH-900</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>NID-1011</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>child</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>10</v>
+      </c>
+      <c r="F33" t="b">
+        <v>1</v>
+      </c>
+      <c r="G33" t="inlineStr">
         <is>
           <t>none</t>
         </is>
@@ -2220,7 +2287,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2264,6 +2331,11 @@
           <t>enrolled_on</t>
         </is>
       </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>observed_at</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -2302,6 +2374,11 @@
       <c r="H2" s="1" t="n">
         <v>45658</v>
       </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>2026-06-19T06:11:12Z</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2340,6 +2417,11 @@
       <c r="H3" s="1" t="n">
         <v>45352</v>
       </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>2026-06-19T06:11:12Z</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2378,6 +2460,11 @@
       <c r="H4" s="1" t="n">
         <v>45809</v>
       </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>2026-06-19T06:11:12Z</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2416,6 +2503,11 @@
       <c r="H5" s="1" t="n">
         <v>45884</v>
       </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>2026-06-19T06:11:12Z</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2454,6 +2546,11 @@
       <c r="H6" s="1" t="n">
         <v>45698</v>
       </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>2026-06-19T06:11:12Z</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2492,6 +2589,11 @@
       <c r="H7" s="1" t="n">
         <v>45646</v>
       </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>2026-06-19T06:11:12Z</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2530,6 +2632,11 @@
       <c r="H8" s="1" t="n">
         <v>45901</v>
       </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>2026-06-19T06:11:12Z</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2568,6 +2675,11 @@
       <c r="H9" s="1" t="n">
         <v>45751</v>
       </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>2026-06-19T06:11:12Z</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2606,6 +2718,11 @@
       <c r="H10" s="1" t="n">
         <v>45778</v>
       </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>2026-06-19T06:11:12Z</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2644,6 +2761,50 @@
       <c r="H11" s="1" t="n">
         <v>45778</v>
       </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>2026-06-17T06:11:12Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>ENR-1011</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>HH-900</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>PER-1011</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>NID-1011</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>CHILD_SUPPORT</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="G12" t="n">
+        <v>85.5</v>
+      </c>
+      <c r="H12" s="1" t="n">
+        <v>45658</v>
+      </c>
+      <c r="I12" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2656,7 +2817,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G32"/>
+  <dimension ref="A1:G33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3621,6 +3782,36 @@
         <v>45658</v>
       </c>
       <c r="G32" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>GM-1011</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>HH-900</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>PER-1011</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>child</t>
+        </is>
+      </c>
+      <c r="E33" s="1" t="n">
+        <v>45658</v>
+      </c>
+      <c r="G33" t="inlineStr">
         <is>
           <t>active</t>
         </is>

</xml_diff>

<commit_message>
Fix evidence gateway lab proof coverage
</commit_message>
<xml_diff>
--- a/data/social-protection/social-protection.xlsx
+++ b/data/social-protection/social-protection.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -471,6 +471,11 @@
           <t>deceased_member_count</t>
         </is>
       </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>observed_at</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -505,6 +510,11 @@
       <c r="H2" t="n">
         <v>0</v>
       </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>2026-06-19T12:59:47Z</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -539,6 +549,11 @@
       <c r="H3" t="n">
         <v>0</v>
       </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>2026-06-19T12:59:47Z</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -573,6 +588,11 @@
       <c r="H4" t="n">
         <v>1</v>
       </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>2026-06-19T12:59:47Z</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -607,6 +627,11 @@
       <c r="H5" t="n">
         <v>0</v>
       </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>2026-06-19T12:59:47Z</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -641,6 +666,11 @@
       <c r="H6" t="n">
         <v>0</v>
       </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>2026-06-19T12:59:47Z</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -675,6 +705,11 @@
       <c r="H7" t="n">
         <v>0</v>
       </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>2026-06-19T12:59:47Z</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -709,6 +744,11 @@
       <c r="H8" t="n">
         <v>0</v>
       </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>2026-06-19T12:59:47Z</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -743,6 +783,11 @@
       <c r="H9" t="n">
         <v>0</v>
       </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>2026-06-17T12:59:47Z</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -777,6 +822,7 @@
       <c r="H10" t="n">
         <v>0</v>
       </c>
+      <c r="I10" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -789,7 +835,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:K3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -843,6 +889,11 @@
           <t>source_version</t>
         </is>
       </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>observed_at</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -891,6 +942,11 @@
           <t>2025.4</t>
         </is>
       </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>2026-06-19T12:59:47Z</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -937,6 +993,11 @@
       <c r="J3" t="inlineStr">
         <is>
           <t>2025.2</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>2026-06-19T12:59:47Z</t>
         </is>
       </c>
     </row>
@@ -951,7 +1012,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1000,6 +1061,11 @@
           <t>review_due</t>
         </is>
       </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>observed_at</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1041,6 +1107,11 @@
       <c r="I2" s="1" t="n">
         <v>46315</v>
       </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>2026-06-19T12:59:47Z</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1081,6 +1152,11 @@
       </c>
       <c r="I3" s="1" t="n">
         <v>45963</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>2026-06-19T12:59:47Z</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -1180,7 +1256,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G33"/>
+  <dimension ref="A1:H33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1219,6 +1295,11 @@
           <t>disability_status</t>
         </is>
       </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>observed_at</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1252,6 +1333,11 @@
           <t>none</t>
         </is>
       </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>2026-06-19T12:59:47Z</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1285,6 +1371,11 @@
           <t>none</t>
         </is>
       </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>2026-06-19T12:59:47Z</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1318,6 +1409,11 @@
           <t>none</t>
         </is>
       </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>2026-06-19T12:59:47Z</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1351,6 +1447,11 @@
           <t>none</t>
         </is>
       </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>2026-06-19T12:59:47Z</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1384,6 +1485,11 @@
           <t>hearing</t>
         </is>
       </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>2026-06-19T12:59:47Z</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1417,6 +1523,11 @@
           <t>none</t>
         </is>
       </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>2026-06-19T12:59:47Z</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1450,6 +1561,11 @@
           <t>none</t>
         </is>
       </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>2026-06-19T12:59:47Z</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1483,6 +1599,11 @@
           <t>none</t>
         </is>
       </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>2026-06-19T12:59:47Z</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1516,6 +1637,11 @@
           <t>none</t>
         </is>
       </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>2026-06-19T12:59:47Z</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1549,6 +1675,11 @@
           <t>physical</t>
         </is>
       </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>2026-06-19T12:59:47Z</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1582,6 +1713,11 @@
           <t>none</t>
         </is>
       </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>2026-06-19T12:59:47Z</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1615,6 +1751,11 @@
           <t>none</t>
         </is>
       </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>2026-06-19T12:59:47Z</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1648,6 +1789,11 @@
           <t>none</t>
         </is>
       </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>2026-06-19T12:59:47Z</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1681,6 +1827,11 @@
           <t>none</t>
         </is>
       </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>2026-06-19T12:59:47Z</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1714,6 +1865,11 @@
           <t>none</t>
         </is>
       </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>2026-06-19T12:59:47Z</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1747,6 +1903,11 @@
           <t>none</t>
         </is>
       </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>2026-06-19T12:59:47Z</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1780,6 +1941,11 @@
           <t>none</t>
         </is>
       </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>2026-06-19T12:59:47Z</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1813,6 +1979,11 @@
           <t>none</t>
         </is>
       </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>2026-06-19T12:59:47Z</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1846,6 +2017,11 @@
           <t>none</t>
         </is>
       </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>2026-06-19T12:59:47Z</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1879,6 +2055,11 @@
           <t>none</t>
         </is>
       </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>2026-06-19T12:59:47Z</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1912,6 +2093,11 @@
           <t>none</t>
         </is>
       </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>2026-06-19T12:59:47Z</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1945,6 +2131,11 @@
           <t>physical</t>
         </is>
       </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>2026-06-19T12:59:47Z</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1978,6 +2169,11 @@
           <t>none</t>
         </is>
       </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>2026-06-19T12:59:47Z</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2011,6 +2207,11 @@
           <t>none</t>
         </is>
       </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>2026-06-19T12:59:47Z</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2044,6 +2245,11 @@
           <t>none</t>
         </is>
       </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>2026-06-19T12:59:47Z</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2077,6 +2283,11 @@
           <t>none</t>
         </is>
       </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>2026-06-17T12:59:47Z</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2110,6 +2321,11 @@
           <t>none</t>
         </is>
       </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>2026-06-19T12:59:47Z</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2143,6 +2359,11 @@
           <t>none</t>
         </is>
       </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>2026-06-19T12:59:47Z</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2176,6 +2397,11 @@
           <t>none</t>
         </is>
       </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>2026-06-19T12:59:47Z</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2209,6 +2435,11 @@
           <t>none</t>
         </is>
       </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>2026-06-19T12:59:47Z</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2242,6 +2473,11 @@
           <t>none</t>
         </is>
       </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>2026-06-19T12:59:47Z</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2275,6 +2511,7 @@
           <t>none</t>
         </is>
       </c>
+      <c r="H33" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2376,7 +2613,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-06-19T06:11:12Z</t>
+          <t>2026-06-19T12:59:47Z</t>
         </is>
       </c>
     </row>
@@ -2419,7 +2656,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026-06-19T06:11:12Z</t>
+          <t>2026-06-19T12:59:47Z</t>
         </is>
       </c>
     </row>
@@ -2462,7 +2699,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-06-19T06:11:12Z</t>
+          <t>2026-06-19T12:59:47Z</t>
         </is>
       </c>
     </row>
@@ -2505,7 +2742,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-06-19T06:11:12Z</t>
+          <t>2026-06-19T12:59:47Z</t>
         </is>
       </c>
     </row>
@@ -2548,7 +2785,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-06-19T06:11:12Z</t>
+          <t>2026-06-19T12:59:47Z</t>
         </is>
       </c>
     </row>
@@ -2591,7 +2828,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-06-19T06:11:12Z</t>
+          <t>2026-06-19T12:59:47Z</t>
         </is>
       </c>
     </row>
@@ -2634,7 +2871,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-06-19T06:11:12Z</t>
+          <t>2026-06-19T12:59:47Z</t>
         </is>
       </c>
     </row>
@@ -2677,7 +2914,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-06-19T06:11:12Z</t>
+          <t>2026-06-19T12:59:47Z</t>
         </is>
       </c>
     </row>
@@ -2720,7 +2957,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-06-19T06:11:12Z</t>
+          <t>2026-06-19T12:59:47Z</t>
         </is>
       </c>
     </row>
@@ -2763,7 +3000,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-06-17T06:11:12Z</t>
+          <t>2026-06-17T12:59:47Z</t>
         </is>
       </c>
     </row>

</xml_diff>